<commit_message>
Fix: Update category model to match with database
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3417AE5-2E58-4FE4-B39A-D524A5FB20D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5677C999-C390-4A7A-A6DE-545DFBDD63C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{24A6269A-75E3-426C-A926-56F40F8FCE69}"/>
+    <workbookView xWindow="11304" yWindow="768" windowWidth="11736" windowHeight="11100" activeTab="1" xr2:uid="{24A6269A-75E3-426C-A926-56F40F8FCE69}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="341">
   <si>
     <t>Name</t>
   </si>
@@ -1028,6 +1028,27 @@
   </si>
   <si>
     <t>Máy lọc không khí LG PuriCare 360 Hit AS60GHWG0 sở hữu thiết kế hiện đại và sang trọng với tông màu thanh lịch, phù hợp với mọi không gian nội thất.</t>
+  </si>
+  <si>
+    <t>C001</t>
+  </si>
+  <si>
+    <t>C002</t>
+  </si>
+  <si>
+    <t>C003</t>
+  </si>
+  <si>
+    <t>C004</t>
+  </si>
+  <si>
+    <t>C005</t>
+  </si>
+  <si>
+    <t>C006</t>
+  </si>
+  <si>
+    <t>C007</t>
   </si>
 </sst>
 </file>
@@ -1414,76 +1435,101 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B14E0942-7384-4F35-A65E-FDB84D1EBF78}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.77734375" customWidth="1"/>
-    <col min="3" max="3" width="9.77734375" customWidth="1"/>
-    <col min="4" max="4" width="121.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.77734375" customWidth="1"/>
+    <col min="4" max="4" width="9.77734375" customWidth="1"/>
+    <col min="5" max="5" width="121.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>334</v>
+      </c>
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>335</v>
+      </c>
+      <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>336</v>
+      </c>
+      <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>337</v>
+      </c>
+      <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>338</v>
+      </c>
+      <c r="B6" t="s">
         <v>15</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>339</v>
+      </c>
+      <c r="B7" t="s">
         <v>17</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>340</v>
+      </c>
+      <c r="B8" t="s">
         <v>19</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1589,7 +1635,7 @@
         <v>46204</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>31</v>
@@ -1636,7 +1682,7 @@
         <v>46204</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>37</v>
@@ -1683,7 +1729,7 @@
         <v>46204</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>38</v>
@@ -1730,7 +1776,7 @@
         <v>46204</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>39</v>
@@ -1777,7 +1823,7 @@
         <v>46204</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>40</v>
@@ -1824,7 +1870,7 @@
         <v>46204</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>41</v>
@@ -1871,7 +1917,7 @@
         <v>46204</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>42</v>
@@ -1918,7 +1964,7 @@
         <v>46204</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>43</v>
@@ -1965,7 +2011,7 @@
         <v>46204</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>44</v>
@@ -2012,7 +2058,7 @@
         <v>46204</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>45</v>
@@ -2059,7 +2105,7 @@
         <v>46204</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>46</v>
@@ -2106,7 +2152,7 @@
         <v>46204</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>47</v>
@@ -2145,7 +2191,7 @@
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
       <c r="J14" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>48</v>
@@ -2184,7 +2230,7 @@
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
       <c r="J15" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>49</v>
@@ -2223,7 +2269,7 @@
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
       <c r="J16" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>50</v>
@@ -2262,7 +2308,7 @@
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>51</v>
@@ -2301,7 +2347,7 @@
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>52</v>
@@ -2340,7 +2386,7 @@
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K19" s="2" t="s">
         <v>53</v>
@@ -2379,7 +2425,7 @@
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K20" s="2" t="s">
         <v>54</v>
@@ -2418,7 +2464,7 @@
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="2" t="s">
-        <v>7</v>
+        <v>334</v>
       </c>
       <c r="K21" s="2" t="s">
         <v>55</v>
@@ -2465,7 +2511,7 @@
         <v>46204</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>9</v>
+        <v>335</v>
       </c>
       <c r="K22" s="2" t="s">
         <v>130</v>
@@ -2512,7 +2558,7 @@
         <v>46204</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>9</v>
+        <v>335</v>
       </c>
       <c r="K23" s="2" t="s">
         <v>131</v>
@@ -2559,7 +2605,7 @@
         <v>46204</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>9</v>
+        <v>335</v>
       </c>
       <c r="K24" s="2" t="s">
         <v>132</v>
@@ -2606,7 +2652,7 @@
         <v>46204</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>9</v>
+        <v>335</v>
       </c>
       <c r="K25" s="2" t="s">
         <v>133</v>
@@ -2653,7 +2699,7 @@
         <v>46204</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>9</v>
+        <v>335</v>
       </c>
       <c r="K26" s="2" t="s">
         <v>134</v>
@@ -2692,7 +2738,7 @@
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
       <c r="J27" s="2" t="s">
-        <v>9</v>
+        <v>335</v>
       </c>
       <c r="K27" s="2" t="s">
         <v>135</v>
@@ -2731,7 +2777,7 @@
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
       <c r="J28" s="2" t="s">
-        <v>9</v>
+        <v>335</v>
       </c>
       <c r="K28" s="2" t="s">
         <v>136</v>
@@ -2770,7 +2816,7 @@
       <c r="H29" s="4"/>
       <c r="I29" s="4"/>
       <c r="J29" s="2" t="s">
-        <v>9</v>
+        <v>335</v>
       </c>
       <c r="K29" s="2" t="s">
         <v>137</v>
@@ -2809,7 +2855,7 @@
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
       <c r="J30" s="2" t="s">
-        <v>9</v>
+        <v>335</v>
       </c>
       <c r="K30" s="2" t="s">
         <v>138</v>
@@ -2848,7 +2894,7 @@
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
       <c r="J31" s="2" t="s">
-        <v>9</v>
+        <v>335</v>
       </c>
       <c r="K31" s="2" t="s">
         <v>139</v>
@@ -2895,7 +2941,7 @@
         <v>46204</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>11</v>
+        <v>336</v>
       </c>
       <c r="K32" s="2" t="s">
         <v>140</v>
@@ -2942,7 +2988,7 @@
         <v>46204</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>11</v>
+        <v>336</v>
       </c>
       <c r="K33" s="2" t="s">
         <v>141</v>
@@ -2989,7 +3035,7 @@
         <v>46204</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>11</v>
+        <v>336</v>
       </c>
       <c r="K34" s="2" t="s">
         <v>142</v>
@@ -3036,7 +3082,7 @@
         <v>46204</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>11</v>
+        <v>336</v>
       </c>
       <c r="K35" s="2" t="s">
         <v>143</v>
@@ -3083,7 +3129,7 @@
         <v>46204</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>11</v>
+        <v>336</v>
       </c>
       <c r="K36" s="2" t="s">
         <v>144</v>
@@ -3122,7 +3168,7 @@
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
       <c r="J37" s="2" t="s">
-        <v>11</v>
+        <v>336</v>
       </c>
       <c r="K37" s="2" t="s">
         <v>145</v>
@@ -3161,7 +3207,7 @@
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
       <c r="J38" s="2" t="s">
-        <v>11</v>
+        <v>336</v>
       </c>
       <c r="K38" s="2" t="s">
         <v>146</v>
@@ -3200,7 +3246,7 @@
       <c r="H39" s="4"/>
       <c r="I39" s="4"/>
       <c r="J39" s="2" t="s">
-        <v>11</v>
+        <v>336</v>
       </c>
       <c r="K39" s="2" t="s">
         <v>147</v>
@@ -3239,7 +3285,7 @@
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
       <c r="J40" s="2" t="s">
-        <v>11</v>
+        <v>336</v>
       </c>
       <c r="K40" s="2" t="s">
         <v>148</v>
@@ -3278,7 +3324,7 @@
       <c r="H41" s="4"/>
       <c r="I41" s="4"/>
       <c r="J41" s="2" t="s">
-        <v>11</v>
+        <v>336</v>
       </c>
       <c r="K41" s="2" t="s">
         <v>149</v>
@@ -3325,7 +3371,7 @@
         <v>46204</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>13</v>
+        <v>337</v>
       </c>
       <c r="K42" s="2" t="s">
         <v>150</v>
@@ -3372,7 +3418,7 @@
         <v>46204</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>13</v>
+        <v>337</v>
       </c>
       <c r="K43" s="2" t="s">
         <v>151</v>
@@ -3419,7 +3465,7 @@
         <v>46204</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>13</v>
+        <v>337</v>
       </c>
       <c r="K44" s="2" t="s">
         <v>152</v>
@@ -3458,7 +3504,7 @@
       <c r="H45" s="4"/>
       <c r="I45" s="4"/>
       <c r="J45" s="2" t="s">
-        <v>13</v>
+        <v>337</v>
       </c>
       <c r="K45" s="2" t="s">
         <v>153</v>
@@ -3497,7 +3543,7 @@
       <c r="H46" s="4"/>
       <c r="I46" s="4"/>
       <c r="J46" s="2" t="s">
-        <v>13</v>
+        <v>337</v>
       </c>
       <c r="K46" s="2" t="s">
         <v>154</v>
@@ -3544,7 +3590,7 @@
         <v>46204</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>15</v>
+        <v>338</v>
       </c>
       <c r="K47" s="2" t="s">
         <v>155</v>
@@ -3591,7 +3637,7 @@
         <v>46204</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>15</v>
+        <v>338</v>
       </c>
       <c r="K48" s="2" t="s">
         <v>156</v>
@@ -3638,7 +3684,7 @@
         <v>46204</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>15</v>
+        <v>338</v>
       </c>
       <c r="K49" s="2" t="s">
         <v>157</v>
@@ -3677,7 +3723,7 @@
       <c r="H50" s="4"/>
       <c r="I50" s="4"/>
       <c r="J50" s="2" t="s">
-        <v>15</v>
+        <v>338</v>
       </c>
       <c r="K50" s="2" t="s">
         <v>158</v>
@@ -3716,7 +3762,7 @@
       <c r="H51" s="4"/>
       <c r="I51" s="4"/>
       <c r="J51" s="2" t="s">
-        <v>15</v>
+        <v>338</v>
       </c>
       <c r="K51" s="2" t="s">
         <v>159</v>
@@ -3763,7 +3809,7 @@
         <v>46204</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>17</v>
+        <v>339</v>
       </c>
       <c r="K52" s="2" t="s">
         <v>160</v>
@@ -3810,7 +3856,7 @@
         <v>46204</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>17</v>
+        <v>339</v>
       </c>
       <c r="K53" s="2" t="s">
         <v>161</v>
@@ -3857,7 +3903,7 @@
         <v>46204</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>17</v>
+        <v>339</v>
       </c>
       <c r="K54" s="2" t="s">
         <v>162</v>
@@ -3896,7 +3942,7 @@
       <c r="H55" s="4"/>
       <c r="I55" s="4"/>
       <c r="J55" s="2" t="s">
-        <v>17</v>
+        <v>339</v>
       </c>
       <c r="K55" s="2" t="s">
         <v>163</v>
@@ -3935,7 +3981,7 @@
       <c r="H56" s="4"/>
       <c r="I56" s="4"/>
       <c r="J56" s="2" t="s">
-        <v>17</v>
+        <v>339</v>
       </c>
       <c r="K56" s="2" t="s">
         <v>164</v>
@@ -3982,7 +4028,7 @@
         <v>46204</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>19</v>
+        <v>340</v>
       </c>
       <c r="K57" s="2" t="s">
         <v>165</v>
@@ -4029,7 +4075,7 @@
         <v>46204</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>19</v>
+        <v>340</v>
       </c>
       <c r="K58" s="2" t="s">
         <v>166</v>
@@ -4076,7 +4122,7 @@
         <v>46204</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>19</v>
+        <v>340</v>
       </c>
       <c r="K59" s="2" t="s">
         <v>167</v>
@@ -4115,7 +4161,7 @@
       <c r="H60" s="4"/>
       <c r="I60" s="4"/>
       <c r="J60" s="2" t="s">
-        <v>19</v>
+        <v>340</v>
       </c>
       <c r="K60" s="2" t="s">
         <v>168</v>
@@ -4154,7 +4200,7 @@
       <c r="H61" s="4"/>
       <c r="I61" s="4"/>
       <c r="J61" s="2" t="s">
-        <v>19</v>
+        <v>340</v>
       </c>
       <c r="K61" s="2" t="s">
         <v>169</v>

</xml_diff>